<commit_message>
Write opaque ARGB colors (FF alpha) so fills render in Excel 2019
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011zPXo8Q6tN5EmphoLMbJyd
</commit_message>
<xml_diff>
--- a/Excel_Test.xlsx
+++ b/Excel_Test.xlsx
@@ -55,70 +55,70 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -437,7 +437,7 @@
     <row r="3">
       <c r="A3">
         <f>A2+B2</f>
-        <v>30</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>